<commit_message>
Update data input - reduce kolom yang tidak perlu
</commit_message>
<xml_diff>
--- a/Data Input/LDM.xlsx
+++ b/Data Input/LDM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://icrafcifor-my.sharepoint.com/personal/d_bodro_landscapealliance_org/Documents/dw/ICRAF/analisis data/CIFOR-ICRAF indonesia/Solusi/Jawa Tengah/0_Regional Ekonomi/R - Regional Ekonomi Jateng/Data Input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{7992EBE8-E815-4178-9BCE-F0D0C86051CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF311354-6FBB-4D22-B574-0FDA963AAB7B}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{7992EBE8-E815-4178-9BCE-F0D0C86051CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C825453F-A24B-4A08-B1DA-92A0BD7F7950}"/>
   <bookViews>
-    <workbookView xWindow="-28935" yWindow="-135" windowWidth="29070" windowHeight="15750" xr2:uid="{353B98BA-F33D-49CB-8D7C-42B1DBC60FEF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{353B98BA-F33D-49CB-8D7C-42B1DBC60FEF}"/>
   </bookViews>
   <sheets>
     <sheet name="LDM" sheetId="1" r:id="rId1"/>
@@ -446,14 +446,14 @@
   <sheetPr>
     <tabColor theme="3" tint="0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:AB67"/>
+  <dimension ref="A1:AA67"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="10.296875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="70.19921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28">
+    <row r="1" spans="1:27">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -535,11 +535,8 @@
       <c r="AA1">
         <v>25</v>
       </c>
-      <c r="AB1">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28">
+    </row>
+    <row r="2" spans="1:27">
       <c r="A2">
         <v>1</v>
       </c>
@@ -621,11 +618,8 @@
       <c r="AA2">
         <v>0</v>
       </c>
-      <c r="AB2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28">
+    </row>
+    <row r="3" spans="1:27">
       <c r="A3">
         <v>2</v>
       </c>
@@ -707,11 +701,8 @@
       <c r="AA3">
         <v>0</v>
       </c>
-      <c r="AB3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28">
+    </row>
+    <row r="4" spans="1:27">
       <c r="A4">
         <v>3</v>
       </c>
@@ -793,11 +784,8 @@
       <c r="AA4">
         <v>0</v>
       </c>
-      <c r="AB4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28">
+    </row>
+    <row r="5" spans="1:27">
       <c r="A5">
         <v>4</v>
       </c>
@@ -879,11 +867,8 @@
       <c r="AA5">
         <v>0</v>
       </c>
-      <c r="AB5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28">
+    </row>
+    <row r="6" spans="1:27">
       <c r="A6">
         <v>5</v>
       </c>
@@ -965,11 +950,8 @@
       <c r="AA6">
         <v>0</v>
       </c>
-      <c r="AB6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28">
+    </row>
+    <row r="7" spans="1:27">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1051,11 +1033,8 @@
       <c r="AA7">
         <v>0</v>
       </c>
-      <c r="AB7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28">
+    </row>
+    <row r="8" spans="1:27">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1137,11 +1116,8 @@
       <c r="AA8">
         <v>0</v>
       </c>
-      <c r="AB8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28">
+    </row>
+    <row r="9" spans="1:27">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1223,11 +1199,8 @@
       <c r="AA9">
         <v>0</v>
       </c>
-      <c r="AB9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28">
+    </row>
+    <row r="10" spans="1:27">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1309,11 +1282,8 @@
       <c r="AA10">
         <v>0</v>
       </c>
-      <c r="AB10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28">
+    </row>
+    <row r="11" spans="1:27">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1395,11 +1365,8 @@
       <c r="AA11">
         <v>0</v>
       </c>
-      <c r="AB11">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28">
+    </row>
+    <row r="12" spans="1:27">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1481,11 +1448,8 @@
       <c r="AA12">
         <v>0</v>
       </c>
-      <c r="AB12">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28">
+    </row>
+    <row r="13" spans="1:27">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1567,11 +1531,8 @@
       <c r="AA13">
         <v>0</v>
       </c>
-      <c r="AB13">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:28">
+    </row>
+    <row r="14" spans="1:27">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1653,11 +1614,8 @@
       <c r="AA14">
         <v>0</v>
       </c>
-      <c r="AB14">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:28">
+    </row>
+    <row r="15" spans="1:27">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1739,11 +1697,8 @@
       <c r="AA15">
         <v>0.1</v>
       </c>
-      <c r="AB15">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:28">
+    </row>
+    <row r="16" spans="1:27">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1825,11 +1780,8 @@
       <c r="AA16">
         <v>0</v>
       </c>
-      <c r="AB16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:28">
+    </row>
+    <row r="17" spans="1:27">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1911,11 +1863,8 @@
       <c r="AA17">
         <v>0</v>
       </c>
-      <c r="AB17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:28">
+    </row>
+    <row r="18" spans="1:27">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1997,11 +1946,8 @@
       <c r="AA18">
         <v>0</v>
       </c>
-      <c r="AB18">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:28">
+    </row>
+    <row r="19" spans="1:27">
       <c r="A19">
         <v>18</v>
       </c>
@@ -2083,11 +2029,8 @@
       <c r="AA19">
         <v>0</v>
       </c>
-      <c r="AB19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:28">
+    </row>
+    <row r="20" spans="1:27">
       <c r="A20">
         <v>19</v>
       </c>
@@ -2169,11 +2112,8 @@
       <c r="AA20">
         <v>0</v>
       </c>
-      <c r="AB20">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:28">
+    </row>
+    <row r="21" spans="1:27">
       <c r="A21">
         <v>20</v>
       </c>
@@ -2255,11 +2195,8 @@
       <c r="AA21">
         <v>0</v>
       </c>
-      <c r="AB21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:28">
+    </row>
+    <row r="22" spans="1:27">
       <c r="A22">
         <v>21</v>
       </c>
@@ -2341,11 +2278,8 @@
       <c r="AA22">
         <v>0</v>
       </c>
-      <c r="AB22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:28">
+    </row>
+    <row r="23" spans="1:27">
       <c r="A23">
         <v>22</v>
       </c>
@@ -2427,11 +2361,8 @@
       <c r="AA23">
         <v>0</v>
       </c>
-      <c r="AB23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:28">
+    </row>
+    <row r="24" spans="1:27">
       <c r="A24">
         <v>23</v>
       </c>
@@ -2513,11 +2444,8 @@
       <c r="AA24">
         <v>0</v>
       </c>
-      <c r="AB24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:28">
+    </row>
+    <row r="25" spans="1:27">
       <c r="A25">
         <v>24</v>
       </c>
@@ -2599,11 +2527,8 @@
       <c r="AA25">
         <v>0</v>
       </c>
-      <c r="AB25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:28">
+    </row>
+    <row r="26" spans="1:27">
       <c r="A26">
         <v>25</v>
       </c>
@@ -2685,11 +2610,8 @@
       <c r="AA26">
         <v>0</v>
       </c>
-      <c r="AB26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:28">
+    </row>
+    <row r="27" spans="1:27">
       <c r="A27">
         <v>26</v>
       </c>
@@ -2771,11 +2693,8 @@
       <c r="AA27">
         <v>0</v>
       </c>
-      <c r="AB27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:28">
+    </row>
+    <row r="28" spans="1:27">
       <c r="A28">
         <v>27</v>
       </c>
@@ -2857,11 +2776,8 @@
       <c r="AA28">
         <v>0</v>
       </c>
-      <c r="AB28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:28">
+    </row>
+    <row r="29" spans="1:27">
       <c r="A29">
         <v>28</v>
       </c>
@@ -2943,11 +2859,8 @@
       <c r="AA29">
         <v>0</v>
       </c>
-      <c r="AB29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:28">
+    </row>
+    <row r="30" spans="1:27">
       <c r="A30">
         <v>29</v>
       </c>
@@ -3029,11 +2942,8 @@
       <c r="AA30">
         <v>0</v>
       </c>
-      <c r="AB30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:28">
+    </row>
+    <row r="31" spans="1:27">
       <c r="A31">
         <v>30</v>
       </c>
@@ -3115,11 +3025,8 @@
       <c r="AA31">
         <v>0</v>
       </c>
-      <c r="AB31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:28">
+    </row>
+    <row r="32" spans="1:27">
       <c r="A32">
         <v>31</v>
       </c>
@@ -3201,11 +3108,8 @@
       <c r="AA32">
         <v>0</v>
       </c>
-      <c r="AB32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:28">
+    </row>
+    <row r="33" spans="1:27">
       <c r="A33">
         <v>32</v>
       </c>
@@ -3287,11 +3191,8 @@
       <c r="AA33">
         <v>0</v>
       </c>
-      <c r="AB33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:28">
+    </row>
+    <row r="34" spans="1:27">
       <c r="A34">
         <v>33</v>
       </c>
@@ -3373,11 +3274,8 @@
       <c r="AA34">
         <v>0</v>
       </c>
-      <c r="AB34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:28">
+    </row>
+    <row r="35" spans="1:27">
       <c r="A35">
         <v>34</v>
       </c>
@@ -3459,11 +3357,8 @@
       <c r="AA35">
         <v>0</v>
       </c>
-      <c r="AB35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:28">
+    </row>
+    <row r="36" spans="1:27">
       <c r="A36">
         <v>35</v>
       </c>
@@ -3545,11 +3440,8 @@
       <c r="AA36">
         <v>0</v>
       </c>
-      <c r="AB36">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:28">
+    </row>
+    <row r="37" spans="1:27">
       <c r="A37">
         <v>36</v>
       </c>
@@ -3631,11 +3523,8 @@
       <c r="AA37">
         <v>0</v>
       </c>
-      <c r="AB37">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:28">
+    </row>
+    <row r="38" spans="1:27">
       <c r="A38">
         <v>37</v>
       </c>
@@ -3717,11 +3606,8 @@
       <c r="AA38">
         <v>0</v>
       </c>
-      <c r="AB38">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:28">
+    </row>
+    <row r="39" spans="1:27">
       <c r="A39">
         <v>38</v>
       </c>
@@ -3803,11 +3689,8 @@
       <c r="AA39">
         <v>0</v>
       </c>
-      <c r="AB39">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:28">
+    </row>
+    <row r="40" spans="1:27">
       <c r="A40">
         <v>39</v>
       </c>
@@ -3889,11 +3772,8 @@
       <c r="AA40">
         <v>0</v>
       </c>
-      <c r="AB40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:28">
+    </row>
+    <row r="41" spans="1:27">
       <c r="A41">
         <v>40</v>
       </c>
@@ -3975,11 +3855,8 @@
       <c r="AA41">
         <v>0</v>
       </c>
-      <c r="AB41">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:28">
+    </row>
+    <row r="42" spans="1:27">
       <c r="A42">
         <v>41</v>
       </c>
@@ -4061,11 +3938,8 @@
       <c r="AA42">
         <v>0</v>
       </c>
-      <c r="AB42">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:28">
+    </row>
+    <row r="43" spans="1:27">
       <c r="A43">
         <v>42</v>
       </c>
@@ -4147,11 +4021,8 @@
       <c r="AA43">
         <v>0</v>
       </c>
-      <c r="AB43">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:28">
+    </row>
+    <row r="44" spans="1:27">
       <c r="A44">
         <v>43</v>
       </c>
@@ -4233,11 +4104,8 @@
       <c r="AA44">
         <v>0</v>
       </c>
-      <c r="AB44">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:28">
+    </row>
+    <row r="45" spans="1:27">
       <c r="A45">
         <v>44</v>
       </c>
@@ -4319,11 +4187,8 @@
       <c r="AA45">
         <v>0</v>
       </c>
-      <c r="AB45">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:28">
+    </row>
+    <row r="46" spans="1:27">
       <c r="A46">
         <v>45</v>
       </c>
@@ -4405,11 +4270,8 @@
       <c r="AA46">
         <v>0</v>
       </c>
-      <c r="AB46">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:28">
+    </row>
+    <row r="47" spans="1:27">
       <c r="A47">
         <v>46</v>
       </c>
@@ -4491,11 +4353,8 @@
       <c r="AA47">
         <v>0</v>
       </c>
-      <c r="AB47">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:28">
+    </row>
+    <row r="48" spans="1:27">
       <c r="A48">
         <v>47</v>
       </c>
@@ -4577,11 +4436,8 @@
       <c r="AA48">
         <v>0</v>
       </c>
-      <c r="AB48">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:28">
+    </row>
+    <row r="49" spans="1:27">
       <c r="A49">
         <v>48</v>
       </c>
@@ -4663,11 +4519,8 @@
       <c r="AA49">
         <v>0</v>
       </c>
-      <c r="AB49">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:28">
+    </row>
+    <row r="50" spans="1:27">
       <c r="A50">
         <v>49</v>
       </c>
@@ -4749,11 +4602,8 @@
       <c r="AA50">
         <v>0</v>
       </c>
-      <c r="AB50">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:28">
+    </row>
+    <row r="51" spans="1:27">
       <c r="A51">
         <v>50</v>
       </c>
@@ -4835,11 +4685,8 @@
       <c r="AA51">
         <v>0</v>
       </c>
-      <c r="AB51">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:28">
+    </row>
+    <row r="52" spans="1:27">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4921,11 +4768,8 @@
       <c r="AA52">
         <v>0</v>
       </c>
-      <c r="AB52">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:28">
+    </row>
+    <row r="53" spans="1:27">
       <c r="A53">
         <v>52</v>
       </c>
@@ -5007,11 +4851,8 @@
       <c r="AA53">
         <v>0</v>
       </c>
-      <c r="AB53">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:28">
+    </row>
+    <row r="54" spans="1:27">
       <c r="A54">
         <v>53</v>
       </c>
@@ -5093,11 +4934,8 @@
       <c r="AA54">
         <v>0</v>
       </c>
-      <c r="AB54">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:28">
+    </row>
+    <row r="55" spans="1:27">
       <c r="A55">
         <v>54</v>
       </c>
@@ -5179,11 +5017,8 @@
       <c r="AA55">
         <v>0</v>
       </c>
-      <c r="AB55">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:28">
+    </row>
+    <row r="56" spans="1:27">
       <c r="A56">
         <v>55</v>
       </c>
@@ -5265,11 +5100,8 @@
       <c r="AA56">
         <v>0</v>
       </c>
-      <c r="AB56">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:28">
+    </row>
+    <row r="57" spans="1:27">
       <c r="A57">
         <v>56</v>
       </c>
@@ -5351,11 +5183,8 @@
       <c r="AA57">
         <v>0</v>
       </c>
-      <c r="AB57">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:28">
+    </row>
+    <row r="58" spans="1:27">
       <c r="A58">
         <v>57</v>
       </c>
@@ -5437,11 +5266,8 @@
       <c r="AA58">
         <v>0</v>
       </c>
-      <c r="AB58">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:28">
+    </row>
+    <row r="59" spans="1:27">
       <c r="A59">
         <v>58</v>
       </c>
@@ -5523,11 +5349,8 @@
       <c r="AA59">
         <v>0</v>
       </c>
-      <c r="AB59">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:28">
+    </row>
+    <row r="60" spans="1:27">
       <c r="A60">
         <v>59</v>
       </c>
@@ -5609,11 +5432,8 @@
       <c r="AA60">
         <v>0</v>
       </c>
-      <c r="AB60">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:28">
+    </row>
+    <row r="61" spans="1:27">
       <c r="A61">
         <v>60</v>
       </c>
@@ -5695,11 +5515,8 @@
       <c r="AA61">
         <v>0</v>
       </c>
-      <c r="AB61">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:28">
+    </row>
+    <row r="62" spans="1:27">
       <c r="A62">
         <v>61</v>
       </c>
@@ -5781,11 +5598,8 @@
       <c r="AA62">
         <v>0</v>
       </c>
-      <c r="AB62">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:28">
+    </row>
+    <row r="63" spans="1:27">
       <c r="A63">
         <v>62</v>
       </c>
@@ -5867,11 +5681,8 @@
       <c r="AA63">
         <v>0</v>
       </c>
-      <c r="AB63">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:28">
+    </row>
+    <row r="64" spans="1:27">
       <c r="A64">
         <v>63</v>
       </c>
@@ -5953,11 +5764,8 @@
       <c r="AA64">
         <v>0</v>
       </c>
-      <c r="AB64">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:28">
+    </row>
+    <row r="65" spans="1:27">
       <c r="A65">
         <v>64</v>
       </c>
@@ -6039,11 +5847,8 @@
       <c r="AA65">
         <v>0</v>
       </c>
-      <c r="AB65">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:28">
+    </row>
+    <row r="66" spans="1:27">
       <c r="A66">
         <v>65</v>
       </c>
@@ -6125,11 +5930,8 @@
       <c r="AA66">
         <v>0</v>
       </c>
-      <c r="AB66">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:28">
+    </row>
+    <row r="67" spans="1:27">
       <c r="A67">
         <v>66</v>
       </c>
@@ -6209,9 +6011,6 @@
         <v>0.9</v>
       </c>
       <c r="AA67">
-        <v>0.9</v>
-      </c>
-      <c r="AB67">
         <v>0.9</v>
       </c>
     </row>

</xml_diff>